<commit_message>
"feat: 升级 process_batch 支持 top_p/frequency_penalty，增加单元测试与性能基准"
</commit_message>
<xml_diff>
--- a/data/reviews_result.xlsx
+++ b/data/reviews_result.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,7 +466,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>质量太差, 三天就坏</t>
+          <t>质量差, 三天就坏</t>
         </is>
       </c>
     </row>
@@ -487,6 +487,66 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>客服态度好, 解决问题快</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>物流速度一般，但东西还不错</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>中性</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>物流速度一般, 东西还不错</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>完全超出预期，性价比超高</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>正面</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>超出预期, 性价比高</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>包装有破损，但内部商品完好</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>中性</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>包装破损, 商品完好</t>
         </is>
       </c>
     </row>

</xml_diff>